<commit_message>
Rebuild pattern, Arabic wordmark, new contact details; redesign quotation, stamps, bag back, footer
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Lrhgz1tp1TUBZWxdySKbKE
</commit_message>
<xml_diff>
--- a/deliverables/05-Quotation/NCL-Quotation-A4-Excel-template.xlsx
+++ b/deliverables/05-Quotation/NCL-Quotation-A4-Excel-template.xlsx
@@ -21,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -99,7 +99,18 @@
       <sz val="8"/>
     </font>
     <font>
+      <name val="Noto Kufi Arabic"/>
+      <b val="1"/>
+      <color rgb="000F1E2A"/>
+      <sz val="8"/>
+    </font>
+    <font>
       <name val="Montserrat"/>
+      <color rgb="0033434F"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Noto Kufi Arabic"/>
       <color rgb="0033434F"/>
       <sz val="8"/>
     </font>
@@ -205,7 +216,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -270,16 +281,24 @@
     <xf numFmtId="4" fontId="11" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1" readingOrder="2"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -390,7 +409,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2114550" cy="381000"/>
+    <ext cx="1143000" cy="209550"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -1173,80 +1192,105 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="26" t="inlineStr">
-        <is>
-          <t>TERMS &amp; CONDITIONS  /  الشروط والأحكام</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="27" t="inlineStr">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>PREPARED BY  /  أعدّه</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>APPROVED BY  /  اعتمده</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>STAMP  /  الختم</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="18" customHeight="1">
+      <c r="A44" s="26" t="n"/>
+      <c r="B44" s="27" t="n"/>
+      <c r="C44" s="26" t="n"/>
+      <c r="D44" s="27" t="n"/>
+      <c r="E44" s="26" t="n"/>
+      <c r="F44" s="27" t="n"/>
+    </row>
+    <row r="45" ht="18" customHeight="1">
+      <c r="A45" s="28" t="n"/>
+      <c r="B45" s="29" t="n"/>
+      <c r="C45" s="28" t="n"/>
+      <c r="D45" s="29" t="n"/>
+      <c r="E45" s="28" t="n"/>
+      <c r="F45" s="29" t="n"/>
+    </row>
+    <row r="46" ht="18" customHeight="1">
+      <c r="A46" s="30" t="n"/>
+      <c r="B46" s="31" t="n"/>
+      <c r="C46" s="30" t="n"/>
+      <c r="D46" s="31" t="n"/>
+      <c r="E46" s="30" t="n"/>
+      <c r="F46" s="31" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="32" t="inlineStr">
+        <is>
+          <t>TERMS &amp; CONDITIONS</t>
+        </is>
+      </c>
+      <c r="D48" s="33" t="inlineStr">
+        <is>
+          <t>الشروط والأحكام</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="30" customHeight="1">
+      <c r="A49" s="34" t="inlineStr">
         <is>
           <t>1. Prices are valid for the period stated above and exclude any taxes or duties not shown.</t>
         </is>
       </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="27" t="inlineStr">
+      <c r="D49" s="35" t="inlineStr">
+        <is>
+          <t>١. الأسعار سارية للمدة المذكورة أعلاه ولا تشمل أي ضرائب أو رسوم غير مبيّنة.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="30" customHeight="1">
+      <c r="A50" s="34" t="inlineStr">
         <is>
           <t>2. Delivery: ____ weeks from order confirmation and receipt of advance payment.</t>
         </is>
       </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="27" t="inlineStr">
+      <c r="D50" s="35" t="inlineStr">
+        <is>
+          <t>٢. التسليم: ____ أسبوعاً من تأكيد الطلب واستلام الدفعة المقدّمة.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="30" customHeight="1">
+      <c r="A51" s="34" t="inlineStr">
         <is>
           <t>3. Warranty: as per the manufacturer's terms for each product supplied.</t>
         </is>
       </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="27" t="inlineStr">
+      <c r="D51" s="35" t="inlineStr">
+        <is>
+          <t>٣. الضمان: وفق شروط الشركة المصنّعة لكل منتج يتم توريده.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="30" customHeight="1">
+      <c r="A52" s="34" t="inlineStr">
         <is>
           <t>4. Any change to the scope or quantities will be quoted separately.</t>
         </is>
       </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="4" t="inlineStr">
-        <is>
-          <t>PREPARED BY  /  أعدّه</t>
-        </is>
-      </c>
-      <c r="C49" s="4" t="inlineStr">
-        <is>
-          <t>APPROVED BY  /  اعتمده</t>
-        </is>
-      </c>
-      <c r="E49" s="4" t="inlineStr">
-        <is>
-          <t>COMPANY STAMP  /  ختم الشركة</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="18" customHeight="1">
-      <c r="A50" s="28" t="n"/>
-      <c r="B50" s="29" t="n"/>
-      <c r="C50" s="28" t="n"/>
-      <c r="D50" s="29" t="n"/>
-      <c r="E50" s="28" t="n"/>
-      <c r="F50" s="29" t="n"/>
-    </row>
-    <row r="51" ht="18" customHeight="1">
-      <c r="A51" s="30" t="n"/>
-      <c r="B51" s="31" t="n"/>
-      <c r="C51" s="30" t="n"/>
-      <c r="D51" s="31" t="n"/>
-      <c r="E51" s="30" t="n"/>
-      <c r="F51" s="31" t="n"/>
-    </row>
-    <row r="52" ht="18" customHeight="1">
-      <c r="A52" s="32" t="n"/>
-      <c r="B52" s="33" t="n"/>
-      <c r="C52" s="32" t="n"/>
-      <c r="D52" s="33" t="n"/>
-      <c r="E52" s="32" t="n"/>
-      <c r="F52" s="33" t="n"/>
+      <c r="D52" s="35" t="inlineStr">
+        <is>
+          <t>٤. أي تغيير في نطاق العمل أو الكميات يُسعَّر بشكل منفصل.</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="4" customHeight="1">
       <c r="A54" s="1" t="n"/>
@@ -1257,58 +1301,64 @@
       <c r="F54" s="1" t="n"/>
     </row>
     <row r="55" ht="17" customHeight="1">
-      <c r="A55" s="34" t="inlineStr">
-        <is>
-          <t>New City Light  ·  Baghdad – Al-Mansour – Al-Dawoodi, Iraq  ·  بغداد – المنصور – الداوودي</t>
+      <c r="A55" s="36" t="inlineStr">
+        <is>
+          <t>New City Light  ·  نيو سيتي لايت  ·  Baghdad, Iraq  ·  بغداد، العراق</t>
         </is>
       </c>
     </row>
     <row r="56" ht="17" customHeight="1">
-      <c r="A56" s="35" t="inlineStr">
-        <is>
-          <t>+964 783 577 6393  ·  +964 786 555 3648  ·  +964 780 517 7717</t>
+      <c r="A56" s="37" t="inlineStr">
+        <is>
+          <t>T  +964 987 654 3210  ·  E  admin@newcitylights.ir  ·  W  www.newcitylights.ir</t>
         </is>
       </c>
     </row>
     <row r="57" ht="17" customHeight="1">
-      <c r="A57" s="35" t="inlineStr">
-        <is>
-          <t>admin@dulights.com  ·  www.dulights.com  ·  LIGHTING THE WAY</t>
+      <c r="A57" s="37" t="inlineStr">
+        <is>
+          <t>LIGHTING THE WAY  ·  إنارة الطريق</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="30">
+  <mergeCells count="36">
     <mergeCell ref="E12:F12"/>
-    <mergeCell ref="A46:F46"/>
     <mergeCell ref="E5:F5"/>
     <mergeCell ref="C14:D14"/>
+    <mergeCell ref="D48:F48"/>
     <mergeCell ref="E14:F14"/>
     <mergeCell ref="A56:F56"/>
+    <mergeCell ref="A50:C50"/>
     <mergeCell ref="A55:F55"/>
     <mergeCell ref="B38:D38"/>
     <mergeCell ref="E8:F8"/>
     <mergeCell ref="A57:F57"/>
     <mergeCell ref="B41:E41"/>
-    <mergeCell ref="A47:F47"/>
     <mergeCell ref="B37:D37"/>
     <mergeCell ref="C10:D10"/>
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="E10:F10"/>
     <mergeCell ref="B40:D40"/>
-    <mergeCell ref="A50:B52"/>
-    <mergeCell ref="C50:D52"/>
+    <mergeCell ref="C44:D46"/>
+    <mergeCell ref="E44:F46"/>
     <mergeCell ref="A12:B12"/>
+    <mergeCell ref="D51:F51"/>
+    <mergeCell ref="A52:C52"/>
     <mergeCell ref="C12:D12"/>
     <mergeCell ref="B36:D36"/>
-    <mergeCell ref="A44:F44"/>
+    <mergeCell ref="D50:F50"/>
     <mergeCell ref="A14:B14"/>
     <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A48:C48"/>
     <mergeCell ref="C8:D8"/>
-    <mergeCell ref="A45:F45"/>
+    <mergeCell ref="A51:C51"/>
+    <mergeCell ref="A49:C49"/>
     <mergeCell ref="A10:B10"/>
-    <mergeCell ref="E50:F52"/>
+    <mergeCell ref="D52:F52"/>
     <mergeCell ref="B39:D39"/>
+    <mergeCell ref="A44:B46"/>
+    <mergeCell ref="D49:F49"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.4" bottom="0.4" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="1" fitToWidth="1"/>

</xml_diff>